<commit_message>
Update RSS and Excel data
</commit_message>
<xml_diff>
--- a/data/国产原创区/国产原创区_titles.xlsx
+++ b/data/国产原创区/国产原创区_titles.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标题清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'标题清单'!$A$1:$A$402</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'标题清单'!$A$1:$A$404</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A402"/>
+  <dimension ref="A1:A404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -461,2812 +461,2826 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>[HD/12.5G]杏吧Up主【探花王安全】原版全集【截至5.9】</t>
+          <t>[FHD/9.61G]【Yisingfeersirb】9.14男女大战 高颜值主播被大屌猛操 bb和奶头都很嫩</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>[4K/FHD/HD/64.8G]大神91Timepasserby 精品丝袜啪啪合集</t>
+          <t>[FHD/11.4G]【tutuya01】9.17-9.18一男战三女 男主轮着干 每个颜值都很高</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>[4K/12.9G]绝美华裔女神asia_fox 高难度动作啪啪</t>
+          <t>[HD/12.5G]杏吧Up主【探花王安全】原版全集【截至5.9】</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>[4K/83.6G]国产新晋长腿白皙极品高颜值网红女优【chloelin520（林千夜Chloe）】4K合集</t>
+          <t>[4K/FHD/HD/64.8G]大神91Timepasserby 精品丝袜啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>[FHD/12.6G]老片新看 调教达人胡子哥大战176瑜伽教练+调教反差人妻姜珂两部合集</t>
+          <t>[4K/12.9G]绝美华裔女神asia_fox 高难度动作啪啪</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>[FHD/51.2G]OF顶级博主 娜娜nana_taipei 25年全集+26年新作</t>
+          <t>[4K/83.6G]国产新晋长腿白皙极品高颜值网红女优【chloelin520（林千夜Chloe）】4K合集</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/63.1G]刘玥 水川瑾 李月如 苏樱花在SpicyGum新片合集【4K修复】</t>
+          <t>[FHD/12.6G]老片新看 调教达人胡子哥大战176瑜伽教练+调教反差人妻姜珂两部合集</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>[FHD/58.6G]国产极品丝袜骚人妻 长腿美乳肥臀御姐【Andmlove】Fansly合集</t>
+          <t>[FHD/51.2G]OF顶级博主 娜娜nana_taipei 25年全集+26年新作</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.19G]网黄超美小姐姐被大屌大力抽插直播小合集</t>
+          <t>[4K/FHD/63.1G]刘玥 水川瑾 李月如 苏樱花在SpicyGum新片合集【4K修复】</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>[FHD/3.99G]91Porn大神【洪荒之力】与模特女友的性爱自拍 孕期也不闲着</t>
+          <t>[FHD/58.6G]国产极品丝袜骚人妻 长腿美乳肥臀御姐【Andmlove】Fansly合集</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/138G]Psychoporn TW「色控&amp;乌托邦」 官方原版大合集</t>
+          <t>[FHD/6.19G]网黄超美小姐姐被大屌大力抽插直播小合集</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>[FHD/56.3G]【探花精品】众探花大神探花各种美女</t>
+          <t>[FHD/3.99G]91Porn大神【洪荒之力】与模特女友的性爱自拍 孕期也不闲着</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>[4K/9.48G]Bunny Miffy 米菲兔《嫂子的诱惑》（第二集）【4K修复】</t>
+          <t>[4K/FHD/138G]Psychoporn TW「色控&amp;乌托邦」 官方原版大合集</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>[FHD/7.82G]51色情短剧《我被困在同一天一千年》全11集</t>
+          <t>[FHD/56.3G]【探花精品】众探花大神探花各种美女</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>[4K/18.1G]国产经典~星空传媒 王拉拉升职记1~3-辰悦</t>
+          <t>[4K/9.48G]Bunny Miffy 米菲兔《嫂子的诱惑》（第二集）【4K修复】</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>[FHD/3.90G]Bunny Miffy 米菲兔 嫂子的诱惑 1+穿连体黑藤丝袜在酒店偷情 OF原版</t>
+          <t>[FHD/7.82G]51色情短剧《我被困在同一天一千年》全11集</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>[FHD/17.6G]【迷人的桃】气质人妻少妇高挑白嫩大长腿黑丝高跟舌吻足交骑乘后入</t>
+          <t>[4K/18.1G]国产经典~星空传媒 王拉拉升职记1~3-辰悦</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.0G]91CM果冻传媒女神「玛丽莲」五部合集【中文字幕】</t>
+          <t>[FHD/3.90G]Bunny Miffy 米菲兔 嫂子的诱惑 1+穿连体黑藤丝袜在酒店偷情 OF原版</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>[4K/21.5G]糖心版 娜娜Nana_taipei新作三部</t>
+          <t>[FHD/17.6G]【迷人的桃】气质人妻少妇高挑白嫩大长腿黑丝高跟舌吻足交骑乘后入</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>[FHD/34.1G]舌吻爆菊舔屄流水无套猛干风骚熟女【草莓味】25年2-4月直播合集</t>
+          <t>[FHD/11.0G]91CM果冻传媒女神「玛丽莲」五部合集【中文字幕】</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>[FHD/30.1G]极品淫妻奶油搅拌器3P~9P啪啪乱交合集</t>
+          <t>[4K/21.5G]糖心版 娜娜Nana_taipei新作三部</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>[FHD/84G]网红极品风骚福利姬NicoLove妮可作品大合集（含P站+OF+糖心）</t>
+          <t>[FHD/34.1G]舌吻爆菊舔屄流水无套猛干风骚熟女【草莓味】25年2-4月直播合集</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>[FHD/17.8G]【维吾尔风情】超大杯白嫩巨乳熟妇性感内衣丝袜旗袍多人运动</t>
+          <t>[FHD/30.1G]极品淫妻奶油搅拌器3P~9P啪啪乱交合集</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>[4K/9.14G]娜娜nana_taipei 「我的邻居是肥臀人妻」新作 OF+糖心版</t>
+          <t>[FHD/84G]网红极品风骚福利姬NicoLove妮可作品大合集（含P站+OF+糖心）</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>[4K/10.1G]超色御姐米菲兔-露全脸新作+饼干姐姐足交自慰新作</t>
+          <t>[FHD/17.8G]【维吾尔风情】超大杯白嫩巨乳熟妇性感内衣丝袜旗袍多人运动</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>[FHD/16.0G]【甜极品奶妈】8月3日-8日、美女被黑人大屌各种姿势狂干</t>
+          <t>[4K/9.14G]娜娜nana_taipei 「我的邻居是肥臀人妻」新作 OF+糖心版</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>[4K/10.6G]【娜娜nana_taipei】封神作~魅魔附身~女老板性癖好测试~办公室勾引男下属肉棒泄欲</t>
+          <t>[4K/10.1G]超色御姐米菲兔-露全脸新作+饼干姐姐足交自慰新作</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>[4K/12.7G]【娜娜nana_taipei】淫荡修女之戴着肛塞渴望肉棒的嫩穴</t>
+          <t>[FHD/16.0G]【甜极品奶妈】8月3日-8日、美女被黑人大屌各种姿势狂干</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>[4K/12.0G]【娜娜nana_taipei】激情通话油亮肉丝被单男疯狂肏穴~打视频出轨给男友看</t>
+          <t>[4K/10.6G]【娜娜nana_taipei】封神作~魅魔附身~女老板性癖好测试~办公室勾引男下属肉棒泄欲</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>[4K/14.8G]【娜娜nana_taipei】痴女太太勾引家里的年轻司机</t>
+          <t>[4K/12.7G]【娜娜nana_taipei】淫荡修女之戴着肛塞渴望肉棒的嫩穴</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>[4K/8.56G]【娜娜nana_taipei】S女王调教家里的公狗，强制射精</t>
+          <t>[4K/12.0G]【娜娜nana_taipei】激情通话油亮肉丝被单男疯狂肏穴~打视频出轨给男友看</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>[4K/10G]娜娜nana_taipei 20240730最新长片 NTR3 给老公的礼物</t>
+          <t>[4K/14.8G]【娜娜nana_taipei】痴女太太勾引家里的年轻司机</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/21.6G]湾湾女优 香蕉电眼女神-狐不妖视频合集</t>
+          <t>[4K/8.56G]【娜娜nana_taipei】S女王调教家里的公狗，强制射精</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>[4K60fps/6.74G]性感优雅御姐新作 BunnyMiffy米菲兔周年祭露脸做爱</t>
+          <t>[4K/10G]娜娜nana_taipei 20240730最新长片 NTR3 给老公的礼物</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>[4K/12.2G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年6月份合集</t>
+          <t>[FHD/HD/21.6G]湾湾女优 香蕉电眼女神-狐不妖视频合集</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>[4K/13.1G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年5月份合集</t>
+          <t>[4K60fps/6.74G]性感优雅御姐新作 BunnyMiffy米菲兔周年祭露脸做爱</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>[4K/13.0G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年4月份合集</t>
+          <t>[4K/12.2G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年6月份合集</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>[4K/11.1G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年3月份合集</t>
+          <t>[4K/13.1G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年5月份合集</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>[4K/14.2G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年2月份合集</t>
+          <t>[4K/13.0G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年4月份合集</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>[4K/11.6G]娜娜nana_taipei 20240708新作 精液搜查官2-驯狗师</t>
+          <t>[4K/11.1G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年3月份合集</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>[4K/18.8G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年1月份合集</t>
+          <t>[4K/14.2G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年2月份合集</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.8G]「国服最强骚话女大学生」听声可射的极品女大小D姐姐</t>
+          <t>[4K/11.6G]娜娜nana_taipei 20240708新作 精液搜查官2-驯狗师</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>[4K/19.8G]娜娜nana_taipei OnlyFans版 灰丝红底高跟的肥美大屁股妈妈被儿子爆操内射</t>
+          <t>[4K/18.8G]台灣第一美乳美臀Ellie ssrpeach（艾莉）2024年1月份合集</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>[4K/14.2G]娜娜nana_taipei OnlyFans版 性感人妻勾引修理工</t>
+          <t>[FHD/13.8G]「国服最强骚话女大学生」听声可射的极品女大小D姐姐</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/12G]糖心版娜娜新作 nana_taipei 富婆攻略手册第二部</t>
+          <t>[4K/19.8G]娜娜nana_taipei OnlyFans版 灰丝红底高跟的肥美大屁股妈妈被儿子爆操内射</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>[4K/35G]早期极品御姐《御姐很哀伤》重制版</t>
+          <t>[4K/14.2G]娜娜nana_taipei OnlyFans版 性感人妻勾引修理工</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>[2K/11.6G]早期上海松江区夫妻自拍流出 重制版</t>
+          <t>[4K/FHD/12G]糖心版娜娜新作 nana_taipei 富婆攻略手册第二部</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.95G]早期网红latour2012年的视频 重制版</t>
+          <t>[4K/35G]早期极品御姐《御姐很哀伤》重制版</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>[4K/25.9G]台湾模特 费爵娜  两部真实啪啪啪！完整无删减</t>
+          <t>[2K/11.6G]早期上海松江区夫妻自拍流出 重制版</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>[4K/4.60G]nana_taipei新作 裸色高跟鞋加肉丝加紫色包臀裙的试穿展示+私信会员视频黑丝</t>
+          <t>[FHD/2.95G]早期网红latour2012年的视频 重制版</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.77G] 糖心VlogUp主【丝袜猫/91t神】合集⭕️猎艳大神⭕️丝袜狂魔⭕️极品丝袜美腿</t>
+          <t>[4K/25.9G]台湾模特 费爵娜  两部真实啪啪啪！完整无删减</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>[FHD/56.4G]极品蜜汁白虎神鲍尤物 娜娜Nana_taipei 糖心Vlog全集</t>
+          <t>[4K/4.60G]nana_taipei新作 裸色高跟鞋加肉丝加紫色包臀裙的试穿展示+私信会员视频黑丝</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>[4K/12G]娜娜新作 nana_taipei2024-05-01 钱债肉偿，只是欠钱就要被干一个下午吗</t>
+          <t>[FHD/8.77G] 糖心VlogUp主【丝袜猫/91t神】合集⭕️猎艳大神⭕️丝袜狂魔⭕️极品丝袜美腿</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>[2K/14.3G]当年火遍全网的龙口中心医院女护士与税务局干部激情大片</t>
+          <t>[FHD/56.4G]极品蜜汁白虎神鲍尤物 娜娜Nana_taipei 糖心Vlog全集</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.04G]替身网红沈樵绝版剧情片-勾引日军中尉的女人</t>
+          <t>[4K/12G]娜娜新作 nana_taipei2024-05-01 钱债肉偿，只是欠钱就要被干一个下午吗</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>[FHD/10.4G]麻豆传媒-国产首位越裔极品女优安娜合集</t>
+          <t>[2K/14.3G]当年火遍全网的龙口中心医院女护士与税务局干部激情大片</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>[FHD/27.4G]「国产高颜值女优」袁子仪（杨柳）合集</t>
+          <t>[FHD/2.04G]替身网红沈樵绝版剧情片-勾引日军中尉的女人</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>[4K/79.7G]nana_taipei 娜娜新作合集【4K修复】</t>
+          <t>[FHD/10.4G]麻豆传媒-国产首位越裔极品女优安娜合集</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/78.6G]国产新人OF博主Bunny Miffy（米菲兔） 合集</t>
+          <t>[FHD/27.4G]「国产高颜值女优」袁子仪（杨柳）合集</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>[FHD/50.5G]台湾AV厂商兔子先生官网无水印原档视频合集3</t>
+          <t>[4K/79.7G]nana_taipei 娜娜新作合集【4K修复】</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>[FHD/50.9G]台湾AV厂商兔子先生官网无水印原档视频合集2</t>
+          <t>[4K/FHD/78.6G]国产新人OF博主Bunny Miffy（米菲兔） 合集</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>[FHD/52.2G]台湾AV厂商兔子先生官网无水印原档视频合集1</t>
+          <t>[FHD/50.5G]台湾AV厂商兔子先生官网无水印原档视频合集3</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>[FHD/25.6G]湾湾新媒体 天使映画 9部影片原档视频合集</t>
+          <t>[FHD/50.9G]台湾AV厂商兔子先生官网无水印原档视频合集2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>[4K/76.9G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-3</t>
+          <t>[FHD/52.2G]台湾AV厂商兔子先生官网无水印原档视频合集1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>[4K/56.0G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-2</t>
+          <t>[FHD/25.6G]湾湾新媒体 天使映画 9部影片原档视频合集</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>[4K/47.6G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-1</t>
+          <t>[4K/76.9G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-3</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>[FHD/34G]国产AV主题秀—高跟美腿冲到爆 穿着高跟鞋做爱主题合集</t>
+          <t>[4K/56.0G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-2</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>[4K/7.75G]TZ-117 原神雷电将军COS 月野靜/矢乃かのん(矢乃花音)下马作【原档+4K】</t>
+          <t>[4K/47.6G]湾湾女优的颜值巅峰 4K收藏版 宋雨川合集-1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>[4K/6.59G]JDKR-038 我的痴女家庭教师 矢乃かのん(矢乃花音)下马作【原档+4K】</t>
+          <t>[FHD/34G]国产AV主题秀—高跟美腿冲到爆 穿着高跟鞋做爱主题合集</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>[FHD/5.44G]国产女优-高梨遥香-91制片厂原档合集</t>
+          <t>[4K/7.75G]TZ-117 原神雷电将军COS 月野靜/矢乃かのん(矢乃花音)下马作【原档+4K】</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>[4K/5.35G]HongKongDoll玩偶姐姐近期新作 衝浪少女的碎碎唸+私信三部4K版</t>
+          <t>[4K/6.59G]JDKR-038 我的痴女家庭教师 矢乃かのん(矢乃花音)下马作【原档+4K】</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>[4K/256G]重新整理_Nana_taipei娜娜1~37期合集4K增强版</t>
+          <t>[FHD/5.44G]国产女优-高梨遥香-91制片厂原档合集</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.98G]91大神唐伯虎和鲜嫩美穴00后学妹坏坏女仆的诱惑视频福利</t>
+          <t>[4K/5.35G]HongKongDoll玩偶姐姐近期新作 衝浪少女的碎碎唸+私信三部4K版</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>[4K/48.8G]Onlyfans_Nana_taipei娜娜新作7部合集4K版</t>
+          <t>[4K/256G]重新整理_Nana_taipei娜娜1~37期合集4K增强版</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>[FHD/19.9G]91大神“物是人非”16部高清大作合集</t>
+          <t>[FHD/5.98G]91大神唐伯虎和鲜嫩美穴00后学妹坏坏女仆的诱惑视频福利</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.44G]P站极品大肥逼，极品身材，台湾在读大学生cola酱Cola5277合集</t>
+          <t>[4K/48.8G]Onlyfans_Nana_taipei娜娜新作7部合集4K版</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>[FHD/10.7G]91大神猫先生近期在电报群，发布的高清版本视频合集</t>
+          <t>[FHD/19.9G]91大神“物是人非”16部高清大作合集</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.56G]SAT-0087 狂飙之正义警官深陷大嫂桃色陷阱 RONA、梁佳芯</t>
+          <t>[FHD/2.44G]P站极品大肥逼，极品身材，台湾在读大学生cola酱Cola5277合集</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>[FHD/30.4G]麻豆纯欲女神苏畅最新作品小合集</t>
+          <t>[FHD/10.7G]91大神猫先生近期在电报群，发布的高清版本视频合集</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>[4K/29.2G]Onlyfans_Nana_taipei娜娜新作4部合集4K版</t>
+          <t>[FHD/6.56G]SAT-0087 狂飙之正义警官深陷大嫂桃色陷阱 RONA、梁佳芯</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.62G]去年爆火过的 [健身哥] 14部长中短视频合集</t>
+          <t>[FHD/30.4G]麻豆纯欲女神苏畅最新作品小合集</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.52G]国内主播-古典气质美女22岁哺乳期紫薇小合集</t>
+          <t>[4K/29.2G]Onlyfans_Nana_taipei娜娜新作4部合集4K版</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.18G]Onlyfans_著名大波女神吴梦梦【厕所痴女勾引男同事3P】</t>
+          <t>[FHD/1.62G]去年爆火过的 [健身哥] 14部长中短视频合集</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.38G]Onlyfans_Nana_taipei娜娜无缝开档油亮灰丝-淫语羞辱寸止挑战</t>
+          <t>[FHD/4.52G]国内主播-古典气质美女22岁哺乳期紫薇小合集</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>[FHD/20.8G]国内首部性爱迷你剧《密友》第一季（01集~43集）</t>
+          <t>[FHD/1.18G]Onlyfans_著名大波女神吴梦梦【厕所痴女勾引男同事3P】</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>[HD/7.08G]Onlyfans_Tangbo_hu唐伯虎新作品小合集</t>
+          <t>[FHD/2.38G]Onlyfans_Nana_taipei娜娜无缝开档油亮灰丝-淫语羞辱寸止挑战</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>[4K/10.0G]Onlyfans_Nana_taipei娜娜最新作品3部小合集4K版</t>
+          <t>[FHD/20.8G]国内首部性爱迷你剧《密友》第一季（01集~43集）</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>[4K/12.9G]Onlyfans_HongKongDoll玩偶姐姐最新作品4部小合集4K版</t>
+          <t>[HD/7.08G]Onlyfans_Tangbo_hu唐伯虎新作品小合集</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.32G]Pornhub站国人博主aria_007视频合集</t>
+          <t>[4K/10.0G]Onlyfans_Nana_taipei娜娜最新作品3部小合集4K版</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>[FHD/28.9G]91风月海棠1~9期视频合集</t>
+          <t>[4K/12.9G]Onlyfans_HongKongDoll玩偶姐姐最新作品4部小合集4K版</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.06G]170CM极品美腿尤物被小个子男前后门贯通2小时40分</t>
+          <t>[FHD/5.32G]Pornhub站国人博主aria_007视频合集</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.00G]萝莉社-阿刚-高端外围探花五部合集</t>
+          <t>[FHD/28.9G]91风月海棠1~9期视频合集</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.37G]鬼畜性奴母狗全程露脸电钻玩弄和菊花高潮不断</t>
+          <t>[FHD/6.06G]170CM极品美腿尤物被小个子男前后门贯通2小时40分</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>[FHD/8.17G]刘玥OnlyFans最新视频+峰不二子路边放尿灌肠自慰完整版</t>
+          <t>[FHD/4.00G]萝莉社-阿刚-高端外围探花五部合集</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.23G]HongKongDoll最新1月私信短片1-4</t>
+          <t>[FHD/3.37G]鬼畜性奴母狗全程露脸电钻玩弄和菊花高潮不断</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.08G]老牌网红EllieLi艾栗栗转战OnlyFans小合集</t>
+          <t>[FHD/8.17G]刘玥OnlyFans最新视频+峰不二子路边放尿灌肠自慰完整版</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.7G]极品大长腿OL办公室空挡喷水</t>
+          <t>[FHD/2.23G]HongKongDoll最新1月私信短片1-4</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11G]国产探花系列文轩-七天探花小合集</t>
+          <t>[FHD/6.08G]老牌网红EllieLi艾栗栗转战OnlyFans小合集</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.84G]极品学院派兼职外围女穿着内衣和高端嫖客无套啪啪</t>
+          <t>[FHD/13.7G]极品大长腿OL办公室空挡喷水</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.72G]超级骚货模特艾小青三亚凤凰岛酒店和金主啪啪</t>
+          <t>[FHD/11G]国产探花系列文轩-七天探花小合集</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>[4K/1.91G]国内少妇与土豪酒店近距离大胆拍摄4k超清</t>
+          <t>[FHD/2.84G]极品学院派兼职外围女穿着内衣和高端嫖客无套啪啪</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>[HD/8.38G]糖心-极品身材小魔女【鸡蛋饼】视频合集</t>
+          <t>[FHD/2.72G]超级骚货模特艾小青三亚凤凰岛酒店和金主啪啪</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>[HD/12.6G]七彩平台主播【尤金金】啪啪紫薇喷水合集</t>
+          <t>[4K/1.91G]国内少妇与土豪酒店近距离大胆拍摄4k超清</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>[HD/13.2G]半糖主播 【涩妈妈】狂尿症！天天喝尿！极度淫荡！被草的胡言乱语</t>
+          <t>[HD/8.38G]糖心-极品身材小魔女【鸡蛋饼】视频合集</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>[HD/14.1G]半糖主播 清纯邻家小妹【想要爸爸抱】合集</t>
+          <t>[HD/12.6G]七彩平台主播【尤金金】啪啪紫薇喷水合集</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.2G]探花系列之李寻欢探花175cm大长腿外围8部合集</t>
+          <t>[HD/13.2G]半糖主播 【涩妈妈】狂尿症！天天喝尿！极度淫荡！被草的胡言乱语</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>[FHD/17.5G]P站-糖心-【小水水】各种啪啪紫薇喷水合集</t>
+          <t>[HD/14.1G]半糖主播 清纯邻家小妹【想要爸爸抱】合集</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.3G]国产AV-星空无限传媒系列 依涵合集</t>
+          <t>[FHD/19.2G]探花系列之李寻欢探花175cm大长腿外围8部合集</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>[FHD/47.6G]国产探花系列之瘦子探花眼镜学妹合集</t>
+          <t>[FHD/17.5G]P站-糖心-【小水水】各种啪啪紫薇喷水合集</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>[FHD/3.06G]娜娜（nana_taipei）onlyfans最新作  老师3</t>
+          <t>[FHD/13.3G]国产AV-星空无限传媒系列 依涵合集</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.9G]糖心-美杜莎新作 巨乳模特与摄影师的情色缠绵</t>
+          <t>[FHD/47.6G]国产探花系列之瘦子探花眼镜学妹合集</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>[FHD/17.7G]绝世骚妇潘金莲 扩阴炮机~下蛋 皮鞋酒瓶插穴喷水</t>
+          <t>[FHD/3.06G]娜娜（nana_taipei）onlyfans最新作  老师3</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>[FHD/30.4G]国产探花系列之杏吧小柒探花合集</t>
+          <t>[FHD/1.9G]糖心-美杜莎新作 巨乳模特与摄影师的情色缠绵</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>[FHD/9.70G]Onlyfans【threexpiggy】付费订阅大合集</t>
+          <t>[FHD/17.7G]绝世骚妇潘金莲 扩阴炮机~下蛋 皮鞋酒瓶插穴喷水</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.97G]OnlyFans健身教练YummyKimmy露脸私拍合集</t>
+          <t>[FHD/30.4G]国产探花系列之杏吧小柒探花合集</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.14G]Onlyfans-亚裔网红officialheimi合集</t>
+          <t>[FHD/9.70G]Onlyfans【threexpiggy】付费订阅大合集</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>[FHD/7.25G]OnlyFans百变女神【Misa米砂】私拍视图合集</t>
+          <t>[FHD/5.97G]OnlyFans健身教练YummyKimmy露脸私拍合集</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>[FHD/16.9G]OnlyFans极品S级女神little私拍合集</t>
+          <t>[FHD/4.14G]Onlyfans-亚裔网红officialheimi合集</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>[HD/15G]七彩美女主播【跳舞老师小糖糖】性感诱惑合集</t>
+          <t>[FHD/7.25G]OnlyFans百变女神【Misa米砂】私拍视图合集</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>[HD/5.93G]【幕幕在深圳】漂亮的深圳美女天天被操+道具自慰</t>
+          <t>[FHD/16.9G]OnlyFans极品S级女神little私拍合集</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>[FHD/49.1G]国产探花系列之探花战神利哥合集</t>
+          <t>[HD/15G]七彩美女主播【跳舞老师小糖糖】性感诱惑合集</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>[HD/4.21G]鲜花直播主播【牧夏/苏乔乔/房琪/琪琪ki 】</t>
+          <t>[HD/5.93G]【幕幕在深圳】漂亮的深圳美女天天被操+道具自慰</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>[HD/22.3G]青瑶主播【棉MM/绵mm/绵绵m 】12月26~31合集</t>
+          <t>[FHD/49.1G]国产探花系列之探花战神利哥合集</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>[HD/5.83G]青瑶直播主播【温柔/林妹妹 】1月3.4日</t>
+          <t>[HD/4.21G]鲜花直播主播【牧夏/苏乔乔/房琪/琪琪ki 】</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.88G]台灣美艳轻熟女 小愛 激情上演</t>
+          <t>[HD/22.3G]青瑶主播【棉MM/绵mm/绵绵m 】12月26~31合集</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>[4K/7.96G]Pornhub站新人【k_loves_yana】最新啪啪小合集</t>
+          <t>[HD/5.83G]青瑶直播主播【温柔/林妹妹 】1月3.4日</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.38G]三个女人和两个男人进行了一场激情四射的现场表演</t>
+          <t>[FHD/3.88G]台灣美艳轻熟女 小愛 激情上演</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.68G]巨乳主播【银耳】雪白粉嫩~诱惑满满</t>
+          <t>[4K/7.96G]Pornhub站新人【k_loves_yana】最新啪啪小合集</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.52G]Pornhub站极品小萝莉【樱花小猫】和男友啪啪合集</t>
+          <t>[FHD/3.38G]三个女人和两个男人进行了一场激情四射的现场表演</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>[HD/7.5G]SP站极品美女主播【bandicam】紫薇高潮喷水</t>
+          <t>[FHD/2.68G]巨乳主播【银耳】雪白粉嫩~诱惑满满</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>[HD/8.89G]半糖主播21岁小姐姐啪啪大秀合集</t>
+          <t>[FHD/5.52G]Pornhub站极品小萝莉【樱花小猫】和男友啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>[FHD/33.1G]人气主播绝世颜值御姐汉娜Hana99道具紫薇喷水</t>
+          <t>[HD/7.5G]SP站极品美女主播【bandicam】紫薇高潮喷水</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>[HD/5.8G]SP站美女主播【ANNA102】小合集</t>
+          <t>[HD/8.89G]半糖主播21岁小姐姐啪啪大秀合集</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/18G]CB站美臀主播【007movie】合集</t>
+          <t>[FHD/33.1G]人气主播绝世颜值御姐汉娜Hana99道具紫薇喷水</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>[HD/9.27G]【雅白】G奶御姐~!骚舌舔奶~各种道具~特写自慰~流白浆</t>
+          <t>[HD/5.8G]SP站美女主播【ANNA102】小合集</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>[HD/4.1G]【小海媚】爆乳御姐乳交花式疯狂操B浪叫勾魂合集</t>
+          <t>[FHD/HD/18G]CB站美臀主播【007movie】合集</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/16.2G]台湾美女艺人 -梁佳芯- 合集</t>
+          <t>[HD/9.27G]【雅白】G奶御姐~!骚舌舔奶~各种道具~特写自慰~流白浆</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.8G]真实三甲医院，刚毕业的小护士！清纯美女，极品肥嫩馒头逼超强诱惑</t>
+          <t>[HD/4.1G]【小海媚】爆乳御姐乳交花式疯狂操B浪叫勾魂合集</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.61G]性感小少妇5小时超大阳具紫薇</t>
+          <t>[FHD/HD/16.2G]台湾美女艺人 -梁佳芯- 合集</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>[FHD/21.1G]CB站主播-长发及腰【lo_vely_su】 直播合集</t>
+          <t>[FHD/19.8G]真实三甲医院，刚毕业的小护士！清纯美女，极品肥嫩馒头逼超强诱惑</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.63G]台湾极品巨乳大骚货娃娃 视频图片合集</t>
+          <t>[FHD/6.61G]性感小少妇5小时超大阳具紫薇</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>[FHD/5.64G]极品主播【徐璐鹿】~03年小可爱超反差！</t>
+          <t>[FHD/21.1G]CB站主播-长发及腰【lo_vely_su】 直播合集</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.04G]带大家一起来某花张xx的吃瓜</t>
+          <t>[FHD/8.63G]台湾极品巨乳大骚货娃娃 视频图片合集</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>[FHD/8.08G]美鲍嫩菊、完美身材极品福利姬Tsubaki全套视频照片资源</t>
+          <t>[FHD/5.64G]极品主播【徐璐鹿】~03年小可爱超反差！</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8G]❤️国人COS天花板❤️P站网红博主YuzuKitty（柚子猫）丝袜党福音</t>
+          <t>[FHD/1.04G]带大家一起来某花张xx的吃瓜</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>[FHD/71.9G]探花系列_9总全国探花合集</t>
+          <t>[FHD/8.08G]美鲍嫩菊、完美身材极品福利姬Tsubaki全套视频照片资源</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>[FHD/32.6G]180超长腿日本妹倩倩被泰国小哥大长屌爆操合集</t>
+          <t>[FHD/8G]❤️国人COS天花板❤️P站网红博主YuzuKitty（柚子猫）丝袜党福音</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>[4K/5.22G]惊艳纯情女神，不需要美颜的那种，被爆菊 被深喉</t>
+          <t>[FHD/71.9G]探花系列_9总全国探花合集</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>[4K/1.15G]极品身材_脸红Dearie_ 高铁之旅</t>
+          <t>[FHD/32.6G]180超长腿日本妹倩倩被泰国小哥大长屌爆操合集</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>[4K/8.55G]玩偶姐姐hongkongdoll新作两部</t>
+          <t>[4K/5.22G]惊艳纯情女神，不需要美颜的那种，被爆菊 被深喉</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/19.4G]国产传媒-萝莉社系列37部合集</t>
+          <t>[4K/1.15G]极品身材_脸红Dearie_ 高铁之旅</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>[4K/7.96G]【泄密】PUA大佬勾搭24岁护士人妻无套内射</t>
+          <t>[4K/8.55G]玩偶姐姐hongkongdoll新作两部</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.56G]萝莉社-家访女老师与学生产生争执最后竟被学生内射中出- 糖糖</t>
+          <t>[FHD/HD/19.4G]国产传媒-萝莉社系列37部合集</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>[4K/1.95G]老虎菜原创私房模特系列-极品身材清纯小美女露脸大尺度拍摄</t>
+          <t>[4K/7.96G]【泄密】PUA大佬勾搭24岁护士人妻无套内射</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>[4K/6.8G]onlyfans网红博主Nana最新作-老师家访指导</t>
+          <t>[FHD/2.56G]萝莉社-家访女老师与学生产生争执最后竟被学生内射中出- 糖糖</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.46G]91站唐伯虎&amp;韦小宝近期更新的视频合集</t>
+          <t>[4K/1.95G]老虎菜原创私房模特系列-极品身材清纯小美女露脸大尺度拍摄</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.65G]【极品主播】平台第一女神⭐绿播转黄【熙颜】两年了终于下海</t>
+          <t>[4K/6.8G]onlyfans网红博主Nana最新作-老师家访指导</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>[FHD/27.8G]探花系列之杏吧【大熊探花】01~13</t>
+          <t>[FHD/4.46G]91站唐伯虎&amp;韦小宝近期更新的视频合集</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.26G]门主王大炮电钻炮击！抖音70W粉网红纹身女【卯哥】泄露全资料</t>
+          <t>[FHD/3.65G]【极品主播】平台第一女神⭐绿播转黄【熙颜】两年了终于下海</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>[4K/13.3G]唯美色影师林希威御用嫩模【张馨瑶】超大尺度私拍</t>
+          <t>[FHD/27.8G]探花系列之杏吧【大熊探花】01~13</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.1G]高颜值主播【娜子呀】被男友各种无套爆插合集</t>
+          <t>[FHD/5.26G]门主王大炮电钻炮击！抖音70W粉网红纹身女【卯哥】泄露全资料</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>[FHD/3.00G]推特网红Anaimiya【奶咪】新作品</t>
+          <t>[4K/13.3G]唯美色影师林希威御用嫩模【张馨瑶】超大尺度私拍</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>[FHD/7.49G]国产美女主播FM胸膜【星妍/甜心奶猫酱】诱惑合集</t>
+          <t>[FHD/13.1G]高颜值主播【娜子呀】被男友各种无套爆插合集</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.31G]Onlyfans【yuahentai】付费啪啪资源</t>
+          <t>[FHD/3.00G]推特网红Anaimiya【奶咪】新作品</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.3G]极品长腿女神【美杜莎】最全合集-高清收藏版</t>
+          <t>[FHD/7.49G]国产美女主播FM胸膜【星妍/甜心奶猫酱】诱惑合集</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>[FHD/141G]国产网红主播【貂蝉戏水】各种啪啪大合集</t>
+          <t>[FHD/2.31G]Onlyfans【yuahentai】付费啪啪资源</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>[FHD/20.5G]国产网红主播【双女杯】各种啪啪合集</t>
+          <t>[FHD/8.3G]极品长腿女神【美杜莎】最全合集-高清收藏版</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>[4K/FHD/129.7G]经典重温 曾火遍全网推女郎【艾栗栗】视频图片合集</t>
+          <t>[FHD/141G]国产网红主播【貂蝉戏水】各种啪啪大合集</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>[FHD/10.9G]推特美乳美鲍网红【绮珂珂】合集</t>
+          <t>[FHD/20.5G]国产网红主播【双女杯】各种啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.7G]天生丽质完美伪娘TS 杨丽娜、粥粥合集</t>
+          <t>[4K/FHD/129.7G]经典重温 曾火遍全网推女郎【艾栗栗】视频图片合集</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>[4K/5.62G]高端ACG业界女神爆机少女▌喵小吉▌年终两套视频图片合集</t>
+          <t>[FHD/10.9G]推特美乳美鲍网红【绮珂珂】合集</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>[HD/12.2G]绿播女神~25小时~【香奈奈】超美网红脸~狂撸到爆蛋</t>
+          <t>[FHD/19.7G]天生丽质完美伪娘TS 杨丽娜、粥粥合集</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>[HD/32.7G]国产主播系列 美乳美鲍女神~【兔子子】合集</t>
+          <t>[4K/5.62G]高端ACG业界女神爆机少女▌喵小吉▌年终两套视频图片合集</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>[4K/5.89G]高端ACG业界女神爆机少女▌喵小吉▌两套视频图片合集</t>
+          <t>[HD/12.2G]绿播女神~25小时~【香奈奈】超美网红脸~狂撸到爆蛋</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>[4K/47.8G]私房大神【华仔】原创私拍系列合集</t>
+          <t>[HD/32.7G]国产主播系列 美乳美鲍女神~【兔子子】合集</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>[4K/6.2G]【極品女神❤️頂級網紅】勁爆網紅美女『柚子貓』两部合集</t>
+          <t>[4K/5.89G]高端ACG业界女神爆机少女▌喵小吉▌两套视频图片合集</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>[FHD/166.5G]唐伯虎（江浙沪超人强/韦小宝）多女主合集</t>
+          <t>[4K/47.8G]私房大神【华仔】原创私拍系列合集</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>[FHD/39.5G]国产主播系列 大长腿高颜值主播【清绾】21部合集</t>
+          <t>[4K/6.2G]【極品女神❤️頂級網紅】勁爆網紅美女『柚子貓』两部合集</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.3G]龙哥岳母来袭 双飞乱伦岳母和媳妇</t>
+          <t>[FHD/166.5G]唐伯虎（江浙沪超人强/韦小宝）多女主合集</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>[FHD/9.52G]超高颜值御姐9分颜值9分身材紫薇合集</t>
+          <t>[FHD/39.5G]国产主播系列 大长腿高颜值主播【清绾】21部合集</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>[HD/12.7G]国产主播系列-双飞名场面8部合集</t>
+          <t>[FHD/6.3G]龙哥岳母来袭 双飞乱伦岳母和媳妇</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.2G]易直播《谜丝媛媛》美足美腿福利 足交 淫语 紫薇</t>
+          <t>[FHD/9.52G]超高颜值御姐9分颜值9分身材紫薇合集</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/9.71G]曾经火爆全网的【采精小蝴蝶】高清修复合集</t>
+          <t>[HD/12.7G]国产主播系列-双飞名场面8部合集</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.47G]170cm九头身御姐！极品美腿！情趣椅子骑乘位，电动玩具抽插</t>
+          <t>[FHD/19.2G]易直播《谜丝媛媛》美足美腿福利 足交 淫语 紫薇</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>[FHD/7.69G]Onlyfans_tangbohu【唐伯虎】订阅视频</t>
+          <t>[FHD/HD/9.71G]曾经火爆全网的【采精小蝴蝶】高清修复合集</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>[FHD/10.3G]国产主播黑丝小骚妇【诗琪】激情5小时</t>
+          <t>[FHD/6.47G]170cm九头身御姐！极品美腿！情趣椅子骑乘位，电动玩具抽插</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>[FHD/11.4G]台湾九头身极品骚货【Nina-chi】Onlyfans福利合集</t>
+          <t>[FHD/7.69G]Onlyfans_tangbohu【唐伯虎】订阅视频</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>[HD/6.76G]中日混血女神【sherry-niko】公主cos装发骚口交滴蜡自慰合集</t>
+          <t>[FHD/10.3G]国产主播黑丝小骚妇【诗琪】激情5小时</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>[FHD/23.8G]国产探花系列之探花返场合集</t>
+          <t>[FHD/11.4G]台湾九头身极品骚货【Nina-chi】Onlyfans福利合集</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.31G]广东小美女【雪梨小可爱】和男友啪啪合集</t>
+          <t>[HD/6.76G]中日混血女神【sherry-niko】公主cos装发骚口交滴蜡自慰合集</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>[FHD/4.23G]大神D先生（EDC）未流出真实啪啪自拍高能完整版</t>
+          <t>[FHD/23.8G]国产探花系列之探花返场合集</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/58.9G]国产探花系列之文轩探花合集</t>
+          <t>[FHD/4.31G]广东小美女【雪梨小可爱】和男友啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>[HD/29.8G]国产探花系列之李寻欢探花合集</t>
+          <t>[FHD/4.23G]大神D先生（EDC）未流出真实啪啪自拍高能完整版</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>[FHD/43.5G]超高颜值小姐姐【甜腻小喵/小乔吃不饱】 一字马打炮内射合集</t>
+          <t>[FHD/HD/58.9G]国产探花系列之文轩探花合集</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>[FHD/66G]MJ精品-覗き魔1-18部精品大合集</t>
+          <t>[HD/29.8G]国产探花系列之李寻欢探花合集</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
         <is>
-          <t>[FHD/62.6G]老虎菜私房原创16弹~25弹+奥特曼1~9弹合集</t>
+          <t>[FHD/43.5G]超高颜值小姐姐【甜腻小喵/小乔吃不饱】 一字马打炮内射合集</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/61.4G]足控福利-wl大心脏合集</t>
+          <t>[FHD/66G]MJ精品-覗き魔1-18部精品大合集</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
         <is>
-          <t>[HD/3.21G]妖女全站终身VIP套图+终身VIP视频7个+露脸相片</t>
+          <t>[FHD/62.6G]老虎菜私房原创16弹~25弹+奥特曼1~9弹合集</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.81G]新人！汉服美女~【四川古典音乐系】道具自慰~好骚好美！</t>
+          <t>[FHD/HD/61.4G]足控福利-wl大心脏合集</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/151G]国产各传媒公司10月合集</t>
+          <t>[HD/3.21G]妖女全站终身VIP套图+终身VIP视频7个+露脸相片</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/10.2G]推特超绝美反差女神『Littlesulaa』啪啪合集</t>
+          <t>[FHD/3.81G]新人！汉服美女~【四川古典音乐系】道具自慰~好骚好美！</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
         <is>
-          <t>[FHD/4.32G]极品黑丝东方航空大长腿空姐</t>
+          <t>[FHD/HD/151G]国产各传媒公司10月合集</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>[FHD/4.97G]私影大神最新第3弹-瑜伽老师粉穴一字马漂亮美乳</t>
+          <t>[FHD/HD/10.2G]推特超绝美反差女神『Littlesulaa』啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
         <is>
-          <t>[FHD/8.36G]PENTHOUS中国首席模特-夏羲瑶-与老公性爱啪啪流出</t>
+          <t>[FHD/4.32G]极品黑丝东方航空大长腿空姐</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/56.1G]【娜娜(nana_taipei)】 至今为止所有视频Onlyfans版</t>
+          <t>[FHD/4.97G]私影大神最新第3弹-瑜伽老师粉穴一字马漂亮美乳</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/9.44G]國產劇情の糖心Vlog✿极品女神『金善雅』合集</t>
+          <t>[FHD/8.36G]PENTHOUS中国首席模特-夏羲瑶-与老公性爱啪啪流出</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>[4K/104G]最顶流の香港网红美少女『HongKongDoll』4K超清合集</t>
+          <t>[FHD/HD/56.1G]【娜娜(nana_taipei)】 至今为止所有视频Onlyfans版</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.95G]【小嘴亲亲】大乱交❤️全是18岁小姑娘三洞齐开❤️妈妈全程高能指挥作战</t>
+          <t>[FHD/HD/9.44G]國產劇情の糖心Vlog✿极品女神『金善雅』合集</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/24.9G]台灣第一女優㊣吳夢夢の原版大合集</t>
+          <t>[4K/104G]最顶流の香港网红美少女『HongKongDoll』4K超清合集</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/4.56G]【P/O双版】applecptv新作-粉内衣肉丝高跟+蓝内衣肉丝高跟</t>
+          <t>[FHD/6.95G]【小嘴亲亲】大乱交❤️全是18岁小姑娘三洞齐开❤️妈妈全程高能指挥作战</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/92.9G]秀人网摄影师果哥资源史上最全合集</t>
+          <t>[FHD/HD/24.9G]台灣第一女優㊣吳夢夢の原版大合集</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
         <is>
-          <t>[FHD/1.61G]applecptv新作*高跟*黑丝*情趣内衣啪啪</t>
+          <t>[FHD/HD/4.56G]【P/O双版】applecptv新作-粉内衣肉丝高跟+蓝内衣肉丝高跟</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.63G]【樱桃小丸子莜】 穿着婚纱激情大战</t>
+          <t>[FHD/HD/92.9G]秀人网摄影师果哥资源史上最全合集</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.73G]P站极品身材国人博主ChineseBunny合集</t>
+          <t>[FHD/1.61G]applecptv新作*高跟*黑丝*情趣内衣啪啪</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>[HD/21.2G]高颜值主播【超级小湿妹】啪啪合集</t>
+          <t>[FHD/3.63G]【樱桃小丸子莜】 穿着婚纱激情大战</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
         <is>
-          <t>[FHD/25G]东南亚高颜值美女主播啪啪合集</t>
+          <t>[FHD/6.73G]P站极品身材国人博主ChineseBunny合集</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>[HD/4.22G]【舔舔达人】一群00后小屁孩群P，场面十分混乱</t>
+          <t>[HD/21.2G]高颜值主播【超级小湿妹】啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
         <is>
-          <t>[HD/1.98G]【玛卡巴卡】美女的毛毛比我头发还浓密</t>
+          <t>[FHD/25G]东南亚高颜值美女主播啪啪合集</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>[FHD/49.4G]Porn hub&amp;OnlyFans&amp;糖心_NaNa-合集</t>
+          <t>[HD/4.22G]【舔舔达人】一群00后小屁孩群P，场面十分混乱</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
         <is>
-          <t>[FHD/106.5G]东南亚泰国水公主、凤凰三姐妹、越南妹合集</t>
+          <t>[HD/1.98G]【玛卡巴卡】美女的毛毛比我头发还浓密</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>[FHD/4.53G]CCAV萝莉社美女雪儿以自己身体讲解性爱知识合集</t>
+          <t>[FHD/49.4G]Porn hub&amp;OnlyFans&amp;糖心_NaNa-合集</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
         <is>
-          <t>[FHD/9.03G]女神糖糖 七部合集</t>
+          <t>[FHD/106.5G]东南亚泰国水公主、凤凰三姐妹、越南妹合集</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>[FHD/30.3G]啪啪类极品主播合集2</t>
+          <t>[FHD/4.53G]CCAV萝莉社美女雪儿以自己身体讲解性爱知识合集</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="inlineStr">
         <is>
-          <t>[FHD/38.3G]啪啪类极品主播合集1</t>
+          <t>[FHD/9.03G]女神糖糖 七部合集</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>[HD/2.36G]TW炮王『信义赵又廷』约炮推特网红Grac婷婷 豪乳纹身</t>
+          <t>[FHD/30.3G]啪啪类极品主播合集2</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="inlineStr">
         <is>
-          <t>[HD/5.10G]推特超骚女神小人妻【猫宝宝】完美版合集</t>
+          <t>[FHD/38.3G]啪啪类极品主播合集1</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>[FHD/44G]国产探花系列精选合集</t>
+          <t>[HD/2.36G]TW炮王『信义赵又廷』约炮推特网红Grac婷婷 豪乳纹身</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="inlineStr">
         <is>
-          <t>[FHD/22.5G]CD小姐姐（叫我嫂子、模特heels）视频合集</t>
+          <t>[HD/5.10G]推特超骚女神小人妻【猫宝宝】完美版合集</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.74G]超极品魅人小妖精黑丝美腿、粉嫩小穴特写、道具自慰高潮</t>
+          <t>[FHD/44G]国产探花系列精选合集</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.82G]最美推特博主『橙醬小甜心/TS-元气美美』大尺度啪啪流出</t>
+          <t>[FHD/22.5G]CD小姐姐（叫我嫂子、模特heels）视频合集</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>[FHD/7.56G]顶级尤物极品身材！纯天然白虎嫩穴</t>
+          <t>[FHD/5.74G]超极品魅人小妖精黑丝美腿、粉嫩小穴特写、道具自慰高潮</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.05G]Onlyfans极品一字马舞蹈练习生yoxi精彩合集</t>
+          <t>[FHD/2.82G]最美推特博主『橙醬小甜心/TS-元气美美』大尺度啪啪流出</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.08G]曾经轰动全网的柳州莫X与男友艳照门事件视图全集</t>
+          <t>[FHD/7.56G]顶级尤物极品身材！纯天然白虎嫩穴</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="inlineStr">
         <is>
-          <t>[FHD/58.6G]台湾色影师Ed Mosaic作品合集</t>
+          <t>[FHD/6.05G]Onlyfans极品一字马舞蹈练习生yoxi精彩合集</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.96G]抖音性感天花板网红【赵一菲】私密流出完整全套</t>
+          <t>[FHD/2.08G]曾经轰动全网的柳州莫X与男友艳照门事件视图全集</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="inlineStr">
         <is>
-          <t>[FHD/18.6G]颜值绝佳舞蹈大学妹子无码露脸合集</t>
+          <t>[FHD/58.6G]台湾色影师Ed Mosaic作品合集</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>[FHD/11.6G]Pornhub@COCONEY 捷克小情侣视频合集</t>
+          <t>[FHD/2.96G]抖音性感天花板网红【赵一菲】私密流出完整全套</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="inlineStr">
         <is>
-          <t>[FHD/22.3G]Pornhub@CloseUpFantasy近距离拍摄抽插</t>
+          <t>[FHD/18.6G]颜值绝佳舞蹈大学妹子无码露脸合集</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.61G]Onlyfans【Saerosoh】臀控福利，后入视角爱好者</t>
+          <t>[FHD/11.6G]Pornhub@COCONEY 捷克小情侣视频合集</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="inlineStr">
         <is>
-          <t>[HD/44.9G]直播探花原版无水印合集2／20201205录制</t>
+          <t>[FHD/22.3G]Pornhub@CloseUpFantasy近距离拍摄抽插</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>[HD/42.9G]直播探花原版无水印合集／20201204录制</t>
+          <t>[FHD/8.61G]Onlyfans【Saerosoh】臀控福利，后入视角爱好者</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/35G]【七天极品探花】无水印合集</t>
+          <t>[HD/44.9G]直播探花原版无水印合集2／20201205录制</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>[FHD/101G]国内各平台主播小姐姐无水印合集8</t>
+          <t>[HD/42.9G]直播探花原版无水印合集／20201204录制</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="3" t="inlineStr">
         <is>
-          <t>[FHD/147G]国内各平台主播小姐姐无水印合集7</t>
+          <t>[FHD/HD/35G]【七天极品探花】无水印合集</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>[FHD/153G]国内各平台主播小姐姐无水印合集6</t>
+          <t>[FHD/101G]国内各平台主播小姐姐无水印合集8</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="inlineStr">
         <is>
-          <t>[FHD/116G]国内各平台主播小姐姐无水印合集5</t>
+          <t>[FHD/147G]国内各平台主播小姐姐无水印合集7</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>[HD/7.96G]高颜值网红【司雨】露脸合集</t>
+          <t>[FHD/153G]国内各平台主播小姐姐无水印合集6</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="inlineStr">
         <is>
-          <t>[4K/13.4G]七天极品探花-高价网约极品女神一字马超粉嫩鲍鱼完美展示</t>
+          <t>[FHD/116G]国内各平台主播小姐姐无水印合集5</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/179G]国内各平台主播小姐姐合集4</t>
+          <t>[HD/7.96G]高颜值网红【司雨】露脸合集</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="inlineStr">
         <is>
-          <t>[FHD/32.3G]泰国高颜值网红【东南亚小妖精】四女一妖合集</t>
+          <t>[4K/13.4G]七天极品探花-高价网约极品女神一字马超粉嫩鲍鱼完美展示</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>[HD/6.77G]探花小飞哥高端外围高颜值极品女神9部合集</t>
+          <t>[FHD/HD/179G]国内各平台主播小姐姐合集4</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.1G]高颜值极品TS『Ladyboy_name』OnlyFans订阅合集</t>
+          <t>[FHD/32.3G]泰国高颜值网红【东南亚小妖精】四女一妖合集</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>[FHD/105G]国产情色主播原版无水印合集3</t>
+          <t>[HD/6.77G]探花小飞哥高端外围高颜值极品女神9部合集</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="inlineStr">
         <is>
-          <t>[FHD/42.2G]金牌摄影师果哥大尺度美模私拍铂金版系列42部全高清合集</t>
+          <t>[FHD/13.1G]高颜值极品TS『Ladyboy_name』OnlyFans订阅合集</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>[FHD/45.2G]国产情色主播原版无水印合集2</t>
+          <t>[FHD/105G]国产情色主播原版无水印合集3</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.38G]神级超美原创91小魔女完美女友型▌美汁源▌合集</t>
+          <t>[FHD/42.2G]金牌摄影师果哥大尺度美模私拍铂金版系列42部全高清合集</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>[H265/4K/16.1G]香港经典三级片【聊斋艳谭三部曲】4K修复版</t>
+          <t>[FHD/45.2G]国产情色主播原版无水印合集2</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="inlineStr">
         <is>
-          <t>[FHD/18.7G]高颜值丰乳肥臀丰满肉感坦克主播合集</t>
+          <t>[FHD/6.38G]神级超美原创91小魔女完美女友型▌美汁源▌合集</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.84G]唯美人妻原创自拍合集</t>
+          <t>[H265/4K/16.1G]香港经典三级片【聊斋艳谭三部曲】4K修复版</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="inlineStr">
         <is>
-          <t>[FHD/12.9G]巨乳馒头网红【可可冥】合集</t>
+          <t>[FHD/18.7G]高颜值丰乳肥臀丰满肉感坦克主播合集</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>[FHD/12.8G]【孕妇也疯狂】真实孕妇性爱记录 完整全收录几年性爱生活变化</t>
+          <t>[FHD/5.84G]唯美人妻原创自拍合集</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="3" t="inlineStr">
         <is>
-          <t>[FHD/127G]Onlyfans@elisetutu69(谭晓彤)作品合集</t>
+          <t>[FHD/12.9G]巨乳馒头网红【可可冥】合集</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.5G]极品JVID超人气名模 璃奈酱六部合集</t>
+          <t>[FHD/12.8G]【孕妇也疯狂】真实孕妇性爱记录 完整全收录几年性爱生活变化</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
         <is>
-          <t>[FHD/HD/81.9G]国内各平台主播小姐姐合集1</t>
+          <t>[FHD/127G]Onlyfans@elisetutu69(谭晓彤)作品合集</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>[HD/33.1G]国产丝雨系列33部合集</t>
+          <t>[FHD/6.5G]极品JVID超人气名模 璃奈酱六部合集</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="inlineStr">
         <is>
-          <t>[FHD/54.6G]国产主播-高颜值清纯美女 甜心小西柚 合集</t>
+          <t>[FHD/HD/81.9G]国内各平台主播小姐姐合集1</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>[FHD/161G]高颜值网红美女【球迷的奶球/汝模姬】 合集</t>
+          <t>[HD/33.1G]国产丝雨系列33部合集</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.49G]推特字母圈大佬【荡妇日记】各种调教95反差婊</t>
+          <t>[FHD/54.6G]国产主播-高颜值清纯美女 甜心小西柚 合集</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>[FHD/4.76G]网爆《三年回忆录》小情侣的三年爱爱路程</t>
+          <t>[FHD/161G]高颜值网红美女【球迷的奶球/汝模姬】 合集</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="inlineStr">
         <is>
-          <t>[HD/3.75G]台湾摄影师⭐ED Mosaic⭐花重金约来公司美女职员挑战十个男人</t>
+          <t>[FHD/6.49G]推特字母圈大佬【荡妇日记】各种调教95反差婊</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.03G]国产极品超级美乳-HeyuZhang张贺玉合集</t>
+          <t>[FHD/4.76G]网爆《三年回忆录》小情侣的三年爱爱路程</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.4G]onlyfans-Pornhub亚籍网红YunaTamaGo合集</t>
+          <t>[HD/3.75G]台湾摄影师⭐ED Mosaic⭐花重金约来公司美女职员挑战十个男人</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>[FHD/14.5G]电报群骚母女，女儿19处女合集</t>
+          <t>[FHD/8.03G]国产极品超级美乳-HeyuZhang张贺玉合集</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.6G]外表极清纯 PornHub网红小e 她太会玩了!!</t>
+          <t>[FHD/19.4G]onlyfans-Pornhub亚籍网红YunaTamaGo合集</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.5G]PornHub亚籍网红 李凯莉 Kylee Lee 合集</t>
+          <t>[FHD/14.5G]电报群骚母女，女儿19处女合集</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="3" t="inlineStr">
         <is>
-          <t>[FHD/22.7G]人妖情侣小貓@CathyBBlove(cmbprod)拼刺刀</t>
+          <t>[FHD/11.6G]外表极清纯 PornHub网红小e 她太会玩了!!</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.0G]福利姬@Lepaudam（LepALuli2kVN）嫩妹合集</t>
+          <t>[FHD/13.5G]PornHub亚籍网红 李凯莉 Kylee Lee 合集</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="3" t="inlineStr">
         <is>
-          <t>[4K/80.6G]老虎菜原创私房系列 1~15全集</t>
+          <t>[FHD/22.7G]人妖情侣小貓@CathyBBlove(cmbprod)拼刺刀</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>[FHD/31.5G]91超气质175cm大长腿极品御姐 淑怡 合集</t>
+          <t>[FHD/13.0G]福利姬@Lepaudam（LepALuli2kVN）嫩妹合集</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.83G]推特福利姬【芋圆呀呀】 极品酥胸紫薇合集</t>
+          <t>[4K/80.6G]老虎菜原创私房系列 1~15全集</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>[FHD/9.44G]P站亚裔网红 PAPAXMAMA合集</t>
+          <t>[FHD/31.5G]91超气质175cm大长腿极品御姐 淑怡 合集</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="3" t="inlineStr">
         <is>
-          <t>[FHD/31G]P站网红留学生 LexisCandyShop合集</t>
+          <t>[FHD/6.83G]推特福利姬【芋圆呀呀】 极品酥胸紫薇合集</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>[FHD/89.8G]Onlyfans_HongKongDOLL合集</t>
+          <t>[FHD/9.44G]P站亚裔网红 PAPAXMAMA合集</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="3" t="inlineStr">
         <is>
-          <t>[FHD/5.14G]【蕾丝兔宝宝】2011-2016全套无修正合集</t>
+          <t>[FHD/31G]P站网红留学生 LexisCandyShop合集</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>[4K/140G]拳交女王【周晓琳】80部合集</t>
+          <t>[FHD/89.8G]Onlyfans_HongKongDOLL合集</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="3" t="inlineStr">
         <is>
-          <t>[4K/5.76G]老虎菜原创私房系列 公司楼梯间口交,操时给男友打电话可惜没接</t>
+          <t>[FHD/5.14G]【蕾丝兔宝宝】2011-2016全套无修正合集</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>[HD/31.3G]东宫媚娘20部视频合集【AI修复】</t>
+          <t>[4K/140G]拳交女王【周晓琳】80部合集</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="3" t="inlineStr">
         <is>
-          <t>[4K/94G]【小鸟酱】写真全集 4K终极收藏版</t>
+          <t>[4K/5.76G]老虎菜原创私房系列 公司楼梯间口交,操时给男友打电话可惜没接</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.3G]推特极品网红【小鹿酱 WJSGMN】合集</t>
+          <t>[HD/31.3G]东宫媚娘20部视频合集【AI修复】</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="3" t="inlineStr">
         <is>
-          <t>[4K/24.8G]91新晋大神【Timepasserby】合集HD增强版</t>
+          <t>[4K/94G]【小鸟酱】写真全集 4K终极收藏版</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.73G]91高清牛哥合集</t>
+          <t>[FHD/13.3G]推特极品网红【小鹿酱 WJSGMN】合集</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="3" t="inlineStr">
         <is>
-          <t>[FHD/35.1G]唐安琪秀人网全高清视图合集</t>
+          <t>[4K/24.8G]91新晋大神【Timepasserby】合集HD增强版</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/74.4G]抖娘-利世图萌社全高清视图合集</t>
+          <t>[FHD/3.73G]91高清牛哥合集</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="3" t="inlineStr">
         <is>
-          <t>[FHD/14.8G]【StripChat】超级女神【sulys】3月天价付费秀喷水紫薇合集</t>
+          <t>[FHD/35.1G]唐安琪秀人网全高清视图合集</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>[FHD/9.87G]推特女神 〖峰不二子〗大尺度私拍流出合集</t>
+          <t>[4K/FHD/74.4G]抖娘-利世图萌社全高清视图合集</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.7G]⭐推特极品女神反差婊⭐爱丝袜的Vivian姐合集</t>
+          <t>[FHD/14.8G]【StripChat】超级女神【sulys】3月天价付费秀喷水紫薇合集</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>[FHD/19.0G]【初恋的香味】极品姐妹花 萝莉御姐极品身材合集</t>
+          <t>[FHD/9.87G]推特女神 〖峰不二子〗大尺度私拍流出合集</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="3" t="inlineStr">
         <is>
-          <t>[FHD/60.9G]半糖主播【一日女友】合集</t>
+          <t>[FHD/13.7G]⭐推特极品女神反差婊⭐爱丝袜的Vivian姐合集</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>[FHD/59.7G]半糖⭐悠悠子⭐“肏”凡大湿--国服第二女喷子</t>
+          <t>[FHD/19.0G]【初恋的香味】极品姐妹花 萝莉御姐极品身材合集</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="3" t="inlineStr">
         <is>
-          <t>[FHD/80.5G]半糖⭐尼尼子⭐“嘴”强王者--国服第一女喷子</t>
+          <t>[FHD/60.9G]半糖主播【一日女友】合集</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>[FHD/10.7G]极品网红『梦菲桐香』土豪订制私拍流出 极致诱惑合集</t>
+          <t>[FHD/59.7G]半糖⭐悠悠子⭐“肏”凡大湿--国服第二女喷子</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="3" t="inlineStr">
         <is>
-          <t>[FHD/20.0G]〖挑战全网喷水最多〗爆裂黑丝潮吹女皇大喷射合集</t>
+          <t>[FHD/80.5G]半糖⭐尼尼子⭐“嘴”强王者--国服第一女喷子</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>[4K/FHD/8.77G]大虎神原创_素人女神合集</t>
+          <t>[FHD/10.7G]极品网红『梦菲桐香』土豪订制私拍流出 极致诱惑合集</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="3" t="inlineStr">
         <is>
-          <t>[FHD/150G]91風吟鳥唱、鳳鳴鳥唱系列大合集</t>
+          <t>[FHD/20.0G]〖挑战全网喷水最多〗爆裂黑丝潮吹女皇大喷射合集</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.79G]妈妈调教女儿-颜值性感母女花全程露脸情趣诱惑</t>
+          <t>[4K/FHD/8.77G]大虎神原创_素人女神合集</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.9G]半糖主播【丝丝袜袜】合集</t>
+          <t>[FHD/150G]91風吟鳥唱、鳳鳴鳥唱系列大合集</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>[FHD/10.8G]小妲己【喵喵是个猫/酥酥唯酥酥】合集</t>
+          <t>[FHD/3.79G]妈妈调教女儿-颜值性感母女花全程露脸情趣诱惑</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="3" t="inlineStr">
         <is>
-          <t>[HD/12.4G]天美传媒抖阴旅行射001-014合集</t>
+          <t>[FHD/13.9G]半糖主播【丝丝袜袜】合集</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>[FHD/154G]OnlyFans-Elise【谭晓彤】大合集</t>
+          <t>[FHD/10.8G]小妲己【喵喵是个猫/酥酥唯酥酥】合集</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="3" t="inlineStr">
         <is>
-          <t>[FHD/58.1G]第一耐操小美女【米拉】的性福生活大合集</t>
+          <t>[HD/12.4G]天美传媒抖阴旅行射001-014合集</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>[FHD/865M]【稀缺资源】美乳女神『Jasmine Lei』大尺度视图，美腿酥胸性感美脚</t>
+          <t>[FHD/154G]OnlyFans-Elise【谭晓彤】大合集</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.0G]【榨精少女&amp;不良忍】平台身材天花板高挑长腿萝莉合集</t>
+          <t>[FHD/58.1G]第一耐操小美女【米拉】的性福生活大合集</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>[FHD/22.4G]半糖主播【越南五朵金花】合集</t>
+          <t>[FHD/865M]【稀缺资源】美乳女神『Jasmine Lei』大尺度视图，美腿酥胸性感美脚</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="3" t="inlineStr">
         <is>
-          <t>[FHD/25.2G]半糖女神『上海卓卓』 模特极致身材直播合集</t>
+          <t>[FHD/13.0G]【榨精少女&amp;不良忍】平台身材天花板高挑长腿萝莉合集</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.5G]Pornhub&amp;OnlyFans【yuahentai】合集</t>
+          <t>[FHD/22.4G]半糖主播【越南五朵金花】合集</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.0G]91大神『啪神BEN』 合集</t>
+          <t>[FHD/25.2G]半糖女神『上海卓卓』 模特极致身材直播合集</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>[FHD/4.04G]七彩主播【卖萌希瑞】极品颜值小女神</t>
+          <t>[FHD/13.5G]Pornhub&amp;OnlyFans【yuahentai】合集</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="3" t="inlineStr">
         <is>
-          <t>[FHD/12.8G]七彩主播【18岁梦涵宝贝】合集3</t>
+          <t>[FHD/19.0G]91大神『啪神BEN』 合集</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>[FHD/72.4G]半糖主播【莹莹baby/小母狗好想要】合集</t>
+          <t>[FHD/4.04G]七彩主播【卖萌希瑞】极品颜值小女神</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.1G]最骚主播 性感电臀女王 合集 白嫩肌肤 性感美臀</t>
+          <t>[FHD/12.8G]七彩主播【18岁梦涵宝贝】合集3</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>[FHD/82.9G]【杨洋小妹妹】自慰啪啪肛交扩阴器洗澡修毛喷水合集</t>
+          <t>[FHD/72.4G]半糖主播【莹莹baby/小母狗好想要】合集</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="3" t="inlineStr">
         <is>
-          <t>[FHD/23G]第一美穴18白虎嫩妹 合集</t>
+          <t>[FHD/11.1G]最骚主播 性感电臀女王 合集 白嫩肌肤 性感美臀</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>[FHD/2.45G]前熊猫主播【杜姗姗】土豪万元定制自慰合集</t>
+          <t>[FHD/82.9G]【杨洋小妹妹】自慰啪啪肛交扩阴器洗澡修毛喷水合集</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="3" t="inlineStr">
         <is>
-          <t>[FHD/17.0G]七彩女神『军阀太太』 粉鲍诱惑直播合集</t>
+          <t>[FHD/23G]第一美穴18白虎嫩妹 合集</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>[FHD/43.2G]91秦先生（小鲜肉、乌索普） 稀缺无水印原版</t>
+          <t>[FHD/2.45G]前熊猫主播【杜姗姗】土豪万元定制自慰合集</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="3" t="inlineStr">
         <is>
-          <t>[FHD/15.1G]Pornhub站HornyCocoLove（91女神丝丝）合集</t>
+          <t>[FHD/17.0G]七彩女神『军阀太太』 粉鲍诱惑直播合集</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>[FHD/65.1G]安能辨我是雌雄 国产TS合集</t>
+          <t>[FHD/43.2G]91秦先生（小鲜肉、乌索普） 稀缺无水印原版</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="3" t="inlineStr">
         <is>
-          <t>[FHD/10.8G]小美女【李溪研】带炮友无套内射</t>
+          <t>[FHD/15.1G]Pornhub站HornyCocoLove（91女神丝丝）合集</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>[FHD/3.20G]情色摄影师 L.P.VISION-MIX.MICO-WUDIAISHEYING合集</t>
+          <t>[FHD/65.1G]安能辨我是雌雄 国产TS合集</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.8G]stripchat站极品主播娜娜annvv直播合集</t>
+          <t>[FHD/10.8G]小美女【李溪研】带炮友无套内射</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.81G]钢琴老师有有_熟女的黑丝诱惑合集</t>
+          <t>[FHD/3.20G]情色摄影师 L.P.VISION-MIX.MICO-WUDIAISHEYING合集</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.5G]推特美足sasa的每一天合集</t>
+          <t>[FHD/11.8G]stripchat站极品主播娜娜annvv直播合集</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.82G]Onlyfans网红小姐姐nana精品小合集</t>
+          <t>[FHD/6.81G]钢琴老师有有_熟女的黑丝诱惑合集</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="3" t="inlineStr">
         <is>
-          <t>[FHD/1.32G]⭐91小马哥调教大二学妹⭐挑战在楼道上打炮惊险又刺激完美露脸</t>
+          <t>[FHD/11.5G]推特美足sasa的每一天合集</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.74G]⭐36D顶级美乳小姐姐⭐情趣内衣粉色渔网袜跳蛋塞穴揉搓</t>
+          <t>[FHD/6.82G]Onlyfans网红小姐姐nana精品小合集</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.61G]极品反差婊阴环女【岳欣悦】多P混战 合集</t>
+          <t>[FHD/1.32G]⭐91小马哥调教大二学妹⭐挑战在楼道上打炮惊险又刺激完美露脸</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>[FHD/83.7G]小姨子和姐夫直播合集02</t>
+          <t>[FHD/6.74G]⭐36D顶级美乳小姐姐⭐情趣内衣粉色渔网袜跳蛋塞穴揉搓</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="3" t="inlineStr">
         <is>
-          <t>[FHD/2.44G]温柔型高颜值甜美女神肉丝美腿近距离特写诱惑</t>
+          <t>[FHD/6.61G]极品反差婊阴环女【岳欣悦】多P混战 合集</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>[FHD/48.4G]Onlyfans网红美少女柚子猫 YuzuKitty 合集</t>
+          <t>[FHD/83.7G]小姨子和姐夫直播合集02</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11G]【李娜娜】合集一 极品骚女被男人玩三洞</t>
+          <t>[FHD/2.44G]温柔型高颜值甜美女神肉丝美腿近距离特写诱惑</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>[FHD/70.6G]【极品合集】七天高端外围系列大合集1</t>
+          <t>[FHD/48.4G]Onlyfans网红美少女柚子猫 YuzuKitty 合集</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="3" t="inlineStr">
         <is>
-          <t>[FHD/128G]❤️完具娜美2017-2021年大合集</t>
+          <t>[FHD/11G]【李娜娜】合集一 极品骚女被男人玩三洞</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>[FHD/117G]小姨子和姐夫直播合集01</t>
+          <t>[FHD/70.6G]【极品合集】七天高端外围系列大合集1</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="3" t="inlineStr">
         <is>
-          <t>[FHD/36G]高颜值福利姬白袜袜格罗丫视频合集</t>
+          <t>[FHD/128G]❤️完具娜美2017-2021年大合集</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>[FHD/16.1G]onlyfans韩国网红xoxo_yuri目前最全合集</t>
+          <t>[FHD/117G]小姨子和姐夫直播合集01</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="3" t="inlineStr">
         <is>
-          <t>[FHD/18.1G]红遍全网绝美颜值91女神 ▌不见星空 ▌大合集</t>
+          <t>[FHD/36G]高颜值福利姬白袜袜格罗丫视频合集</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.72G]小狐狸主播【一点甜甜蜜】高颜值尤物【2022年4月21日收费房】</t>
+          <t>[FHD/16.1G]onlyfans韩国网红xoxo_yuri目前最全合集</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="3" t="inlineStr">
         <is>
-          <t>[FHD/5.99G]七彩主播【18岁梦涵宝贝】合集2</t>
+          <t>[FHD/18.1G]红遍全网绝美颜值91女神 ▌不见星空 ▌大合集</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>[FHD/10.9G]OnlyFans-hookup换妻俱乐部极品人妻</t>
+          <t>[FHD/6.72G]小狐狸主播【一点甜甜蜜】高颜值尤物【2022年4月21日收费房】</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="3" t="inlineStr">
         <is>
-          <t>[FHD/12.9G]极品福利姬萌白酱 超级粉嫩合集</t>
+          <t>[FHD/5.99G]七彩主播【18岁梦涵宝贝】合集2</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>[HD/6.79G]大神azxyq真实约炮170舞蹈系学妹系列完整版</t>
+          <t>[FHD/10.9G]OnlyFans-hookup换妻俱乐部极品人妻</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="3" t="inlineStr">
         <is>
-          <t>[FHD/24.7G]Onlyfans百万粉丝网韩国健身教练yummykimmy福利合集</t>
+          <t>[FHD/12.9G]极品福利姬萌白酱 超级粉嫩合集</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>[FHD/24.2G]甜美女神【顶点】清纯校园妹子合集2</t>
+          <t>[HD/6.79G]大神azxyq真实约炮170舞蹈系学妹系列完整版</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.8G]推特大神bbbmwz合集</t>
+          <t>[FHD/24.7G]Onlyfans百万粉丝网韩国健身教练yummykimmy福利合集</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.1G]91系列极品推特人妻『雪玲儿』土豪专享性爱私拍合集</t>
+          <t>[FHD/24.2G]甜美女神【顶点】清纯校园妹子合集2</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11G][Cosplay] 爆机美少女喵小吉合集</t>
+          <t>[FHD/11.8G]推特大神bbbmwz合集</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>[FHD/36.7G]OnlyFans高质量韩国网红@sseu_dam 作品合集</t>
+          <t>[FHD/13.1G]91系列极品推特人妻『雪玲儿』土豪专享性爱私拍合集</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="3" t="inlineStr">
         <is>
-          <t>[FHD/19.3G]91极品萝莉美少女【 粉色情人 】作品大合集</t>
+          <t>[FHD/11G][Cosplay] 爆机美少女喵小吉合集</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>[FHD/16.7G]极品炮台91GD超模現改名69DD合集</t>
+          <t>[FHD/36.7G]OnlyFans高质量韩国网红@sseu_dam 作品合集</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="3" t="inlineStr">
         <is>
-          <t>[FHD/12.4G]推特大神【kimheezkk】3P约啪00后巨乳小母狗合集</t>
+          <t>[FHD/19.3G]91极品萝莉美少女【 粉色情人 】作品大合集</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>[FHD/6.15G]网红主播双阴道的❤️板凳❤️小合集</t>
+          <t>[FHD/16.7G]极品炮台91GD超模現改名69DD合集</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="3" t="inlineStr">
         <is>
-          <t>[FHD/25.6G]OnlyFans韩国极品福利姬【redrose】最全合集(已退圈)</t>
+          <t>[FHD/12.4G]推特大神【kimheezkk】3P约啪00后巨乳小母狗合集</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.56G]福利姬薇薇安vivian最全合集</t>
+          <t>[FHD/6.15G]网红主播双阴道的❤️板凳❤️小合集</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="3" t="inlineStr">
         <is>
-          <t>[FHD/9.42G]甜美女神【顶点】清纯校园妹子</t>
+          <t>[FHD/25.6G]OnlyFans韩国极品福利姬【redrose】最全合集(已退圈)</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>[4K/30.9G]我的幼师女友+林志玲超高清写真套图</t>
+          <t>[FHD/8.56G]福利姬薇薇安vivian最全合集</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="3" t="inlineStr">
         <is>
-          <t>[FHD/3.07G]顶级摄影女神『丝蓓绮』超唯美色影流出 美乳粉穴</t>
+          <t>[FHD/9.42G]甜美女神【顶点】清纯校园妹子</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>[FHD/20.5G]七彩主播【18岁梦涵宝贝】合集</t>
+          <t>[4K/30.9G]我的幼师女友+林志玲超高清写真套图</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="3" t="inlineStr">
         <is>
-          <t>[FHD/69.5G]丝足福利b站丝足asmr大小姐金克丝jinx定制合集</t>
+          <t>[FHD/3.07G]顶级摄影女神『丝蓓绮』超唯美色影流出 美乳粉穴</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>[FHD/8.97G]老资源 超极品《御姐很哀伤》图片视频合集</t>
+          <t>[FHD/20.5G]七彩主播【18岁梦涵宝贝】合集</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="3" t="inlineStr">
         <is>
-          <t>[FHD/13.5G]PornHub站李凯莉 Kylee Lee 合集</t>
+          <t>[FHD/69.5G]丝足福利b站丝足asmr大小姐金克丝jinx定制合集</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>[FHD/17.2G]台湾露脸小姐姐-Daisybaby R站+P站大合集</t>
+          <t>[FHD/8.97G]老资源 超极品《御姐很哀伤》图片视频合集</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="3" t="inlineStr">
         <is>
-          <t>[FHD/11.6G]⭐稀有珍藏⭐稀有模特&lt;murmure&gt;大尺度定制套图视频三点全露</t>
+          <t>[FHD/13.5G]PornHub站李凯莉 Kylee Lee 合集</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>[FHD/5.31G]onlyfans-everyallday 福利姬大胸美乳加白虎男女双吃</t>
+          <t>[FHD/17.2G]台湾露脸小姐姐-Daisybaby R站+P站大合集</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="3" t="inlineStr">
         <is>
-          <t>[HD/11.6G]半塘主播【隔壁小姐姐】神级颜值女神下海直播</t>
+          <t>[FHD/11.6G]⭐稀有珍藏⭐稀有模特&lt;murmure&gt;大尺度定制套图视频三点全露</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.2G]微博美妖张思妮视频合集</t>
+          <t>[FHD/5.31G]onlyfans-everyallday 福利姬大胸美乳加白虎男女双吃</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="3" t="inlineStr">
         <is>
-          <t>[FHD/9.77G]推特TS曦曦（xixiyaxixi1）黑丝、制服系列合集</t>
+          <t>[HD/11.6G]半塘主播【隔壁小姐姐】神级颜值女神下海直播</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>[FHD/13.9G]推特13万粉丝网红TS CDXUN Onlyfans 福利合集</t>
+          <t>[FHD/13.2G]微博美妖张思妮视频合集</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="3" t="inlineStr">
         <is>
-          <t>[FHD/31.2G]【稀有绝版】就是阿朱啊合集</t>
+          <t>[FHD/9.77G]推特TS曦曦（xixiyaxixi1）黑丝、制服系列合集</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>[FHD/44.6G]半糖网红主播合集</t>
+          <t>[FHD/13.9G]推特13万粉丝网红TS CDXUN Onlyfans 福利合集</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="3" t="inlineStr">
         <is>
-          <t>[FHD/33.5G]推特网红Anaimiya奶咪合集</t>
+          <t>[FHD/31.2G]【稀有绝版】就是阿朱啊合集</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>[HD/24.9G]极品尤物漂亮黄毛妹妹合集</t>
+          <t>[FHD/44.6G]半糖网红主播合集</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="3" t="inlineStr">
         <is>
-          <t>[HD/14.2G]刷新三观 母子直播秀场合集</t>
+          <t>[FHD/33.5G]推特网红Anaimiya奶咪合集</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>[HD/43.5G]刷新三观 母女直播秀场合集</t>
+          <t>[HD/24.9G]极品尤物漂亮黄毛妹妹合集</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="3" t="inlineStr">
         <is>
-          <t>[FHD/20.1G]爆乳粉鲍Shiroissad Onlyfans合集</t>
+          <t>[HD/14.2G]刷新三观 母子直播秀场合集</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>[HD/FHD/176G]果冻传媒91CM大合集</t>
+          <t>[HD/43.5G]刷新三观 母女直播秀场合集</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="3" t="inlineStr">
         <is>
-          <t>[4K/2.32G]⭐大长腿超正人体模特【李黎】4K画质原版</t>
+          <t>[FHD/20.1G]爆乳粉鲍Shiroissad Onlyfans合集</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.30G]⭐JVID最强腿神⭐『小蝶』⭐黑丝网袜勾人心魄</t>
+          <t>[HD/FHD/176G]果冻传媒91CM大合集</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.01G]JVID女神⭐SSS级尤物 神鲍美乳&lt;璃奈酱&gt;沈娜娜合集</t>
+          <t>[4K/2.32G]⭐大长腿超正人体模特【李黎】4K画质原版</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>[HD/1.78G]⭐真正的骚货来袭！2小时不间断性爱，高潮水流一地</t>
+          <t>[FHD/1.30G]⭐JVID最强腿神⭐『小蝶』⭐黑丝网袜勾人心魄</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="3" t="inlineStr">
         <is>
-          <t>[FHD/1.46G]⭐超极品91新晋SSS极品尤物⭐MissA⭐第二弹</t>
+          <t>[FHD/6.01G]JVID女神⭐SSS级尤物 神鲍美乳&lt;璃奈酱&gt;沈娜娜合集</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>[FHD/1.43G]⭐超极品91新晋SSS极品尤物⭐MissA⭐第一弹</t>
+          <t>[HD/1.78G]⭐真正的骚货来袭！2小时不间断性爱，高潮水流一地</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="3" t="inlineStr">
         <is>
-          <t>[HD/2.48G]⭐白嫖Miumiu⭐未流出系列</t>
+          <t>[FHD/1.46G]⭐超极品91新晋SSS极品尤物⭐MissA⭐第二弹</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>[HD/6.36G]蜜桃传媒MTCM.唐茜合集</t>
+          <t>[FHD/1.43G]⭐超极品91新晋SSS极品尤物⭐MissA⭐第一弹</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="3" t="inlineStr">
         <is>
-          <t>[HD/5.93G]⭐高端泄密⭐推特女神@女友潇潇完整版档案泄密</t>
+          <t>[HD/2.48G]⭐白嫖Miumiu⭐未流出系列</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>[HD/41.3G]⭐最强淫语⭐《桃谷谷》各种丝袜制服诱惑合集</t>
+          <t>[HD/6.36G]蜜桃传媒MTCM.唐茜合集</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="3" t="inlineStr">
         <is>
-          <t>[FHD/85.9G]⭐半糖主播⭐ 眼镜美女⭐欲姐姐⭐合集</t>
+          <t>[HD/5.93G]⭐高端泄密⭐推特女神@女友潇潇完整版档案泄密</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>[HD/27.1G]星空传媒XKCM.Collection</t>
+          <t>[HD/41.3G]⭐最强淫语⭐《桃谷谷》各种丝袜制服诱惑合集</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="3" t="inlineStr">
         <is>
-          <t>[FHD/6.59G]♒你的白月光♒大神唐伯虎/韦小宝未流出原档5部</t>
+          <t>[FHD/85.9G]⭐半糖主播⭐ 眼镜美女⭐欲姐姐⭐合集</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>[FHD/HD/12G]糖心up主『小桃』合集</t>
+          <t>[HD/27.1G]星空传媒XKCM.Collection</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="3" t="inlineStr">
         <is>
-          <t>[TS/5.22G]麻豆传媒MD完美女友沈娜娜原档全集</t>
+          <t>[FHD/6.59G]♒你的白月光♒大神唐伯虎/韦小宝未流出原档5部</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
+          <t>[FHD/HD/12G]糖心up主『小桃』合集</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>[TS/5.22G]麻豆传媒MD完美女友沈娜娜原档全集</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
           <t>[FHD/313G]铁JB《利哥探花》大合集</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A402"/>
+  <autoFilter ref="A1:A404"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -3669,6 +3683,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A400" r:id="rId399"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A401" r:id="rId400"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A404" r:id="rId403"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>